<commit_message>
feat: Planning template part1
</commit_message>
<xml_diff>
--- a/reports/Group/Planning-Template.xlsx
+++ b/reports/Group/Planning-Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DPOSM\my\2C\dp2\proyecto\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DPOSM\my\2C\dp2\workspace\Workspace-26\Projects\Acme-Starters-B\reports\Group\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35EFCD65-4D08-4FE8-AA27-9C289B796D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFC2F4F-3145-4B6B-A003-862E26C67CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{683E09B8-1D94-4905-B116-9D998A46AAA3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{683E09B8-1D94-4905-B116-9D998A46AAA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Copyright" sheetId="10" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="207">
   <si>
     <t xml:space="preserve">  Enter configuration data in these cells</t>
   </si>
@@ -593,6 +593,93 @@
   </si>
   <si>
     <t>Check D1 In EV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> L04 – Formal testing-S01 – Functional testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> L04 – Formal testing-S02 – Performance testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> L04 – Formal testing-S03 – Advanced topics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L05 – Miscellaneous topics-S01 – Workshop </t>
+  </si>
+  <si>
+    <t>Workshop Presentations</t>
+  </si>
+  <si>
+    <t>Design the relational model</t>
+  </si>
+  <si>
+    <t>Write questions, possible solutions and chosen option</t>
+  </si>
+  <si>
+    <t>Obtain / update Manager role.</t>
+  </si>
+  <si>
+    <t>Create / list projects.</t>
+  </si>
+  <si>
+    <t>Show and update a project.</t>
+  </si>
+  <si>
+    <t>Add Sample data ( Manager and ProjectSquad ).</t>
+  </si>
+  <si>
+    <t>Implement Dashboard model.</t>
+  </si>
+  <si>
+    <t>Implement Project , Managar , ProjectSquad, components model.</t>
+  </si>
+  <si>
+    <t>Implement banner model, service, controller, UI.</t>
+  </si>
+  <si>
+    <t>Implement sponsorship, auditReport link with project, UI, model, service, controller.</t>
+  </si>
+  <si>
+    <t>Implement list and show projects (Any role).</t>
+  </si>
+  <si>
+    <t>Implement effort and TotalActiveMonths update  (update / publish / delete / assign in components).</t>
+  </si>
+  <si>
+    <t>Delete project.</t>
+  </si>
+  <si>
+    <t>Publish project.</t>
+  </si>
+  <si>
+    <t>Implement list and show Inventios (Project-squad role).</t>
+  </si>
+  <si>
+    <t>List member.</t>
+  </si>
+  <si>
+    <t>List member (Any role).</t>
+  </si>
+  <si>
+    <t>Assign / unlink components.</t>
+  </si>
+  <si>
+    <t>List spokespeople, fundrasisers, inventors thar aren't in the project.</t>
+  </si>
+  <si>
+    <t>List show campaigns, strategies.</t>
+  </si>
+  <si>
+    <t>List show sponsorship, donations.</t>
+  </si>
+  <si>
+    <t>Implement Dashboard service and controller.</t>
+  </si>
+  <si>
+    <t>Add Sample / Error data ( Project and Memeber ).</t>
+  </si>
+  <si>
+    <t>List show auditReport , AuditSection</t>
   </si>
 </sst>
 </file>
@@ -6572,7 +6659,7 @@
       </c>
       <c r="K101" s="45" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="L101" s="47">
         <v>1.87</v>
@@ -6621,7 +6708,7 @@
       </c>
       <c r="K102" s="45" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="L102" s="47">
         <v>0.5</v>
@@ -6670,7 +6757,7 @@
       </c>
       <c r="K103" s="45" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="L103" s="47">
         <v>0.25</v>
@@ -6721,7 +6808,7 @@
       </c>
       <c r="K104" s="45" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="L104" s="47">
         <v>1</v>
@@ -6772,7 +6859,7 @@
       </c>
       <c r="K105" s="45" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="L105" s="47">
         <v>1</v>
@@ -6823,7 +6910,7 @@
       </c>
       <c r="K106" s="45" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="L106" s="47">
         <v>0.33</v>
@@ -7058,7 +7145,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="15" width="18.88671875" customWidth="1"/>
-    <col min="16" max="16" width="64.5546875" customWidth="1"/>
+    <col min="16" max="16" width="96.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
@@ -7122,7 +7209,7 @@
       </c>
       <c r="E6" s="35">
         <f>SUM(N11:N110)</f>
-        <v>0</v>
+        <v>1157.75</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
@@ -7143,7 +7230,7 @@
       </c>
       <c r="E7" s="36">
         <f>SUM(O11:O110)</f>
-        <v>0</v>
+        <v>1146.5</v>
       </c>
       <c r="J7" s="37"/>
     </row>
@@ -7223,30 +7310,48 @@
       </c>
       <c r="C11" s="42" t="str">
         <f>IF(ISBLANK(D11), "", _xlfn.CONCAT("T", TEXT(B11, "0000"), "/", VLOOKUP(D11, Internal!$B$35:C$39, 2, FALSE), IF(OR(D11="QA", D11="Revision"), _xlfn.CONCAT("/", H11), "")))</f>
-        <v/>
-      </c>
-      <c r="D11" s="44"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="44"/>
+        <v>T0001/O</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="44" t="s">
+        <v>30</v>
+      </c>
       <c r="H11" s="43"/>
-      <c r="I11" s="46"/>
-      <c r="J11" s="46"/>
+      <c r="I11" s="46">
+        <v>46118.444444444445</v>
+      </c>
+      <c r="J11" s="46">
+        <v>46118.520833333336</v>
+      </c>
       <c r="K11" s="45" t="str">
         <f ca="1">IF(OR(I11="",J11=""),"",IF(AND(J11&lt;&gt;"",I11&gt;=NOW()),"Planned",IF(AND(J11&lt;&gt;"",J11&lt;NOW()),"Completed","Ongoing")))</f>
-        <v/>
-      </c>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L11" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="M11" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N11" s="45">
         <f>IF(ISBLANK(L11), "", L11*VLOOKUP($F11,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O11" s="45" t="str">
+        <v>0</v>
+      </c>
+      <c r="O11" s="45">
         <f>IF(ISBLANK(M11), "", M11*VLOOKUP($F11,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P11" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="P11" s="44" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="12" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="41">
@@ -7254,30 +7359,48 @@
       </c>
       <c r="C12" s="42" t="str">
         <f>IF(ISBLANK(D12), "", _xlfn.CONCAT("T", TEXT(B12, "0000"), "/", VLOOKUP(D12, Internal!$B$35:C$39, 2, FALSE), IF(OR(D12="QA", D12="Revision"), _xlfn.CONCAT("/", H12), "")))</f>
-        <v/>
-      </c>
-      <c r="D12" s="44"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="44"/>
+        <v>T0002/O</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="44" t="s">
+        <v>30</v>
+      </c>
       <c r="H12" s="43"/>
-      <c r="I12" s="46"/>
-      <c r="J12" s="46"/>
+      <c r="I12" s="46">
+        <v>46121.354166666664</v>
+      </c>
+      <c r="J12" s="46">
+        <v>46121.430555555555</v>
+      </c>
       <c r="K12" s="45" t="str">
         <f t="shared" ref="K12:K75" ca="1" si="0">IF(OR(I12="",J12=""),"",IF(AND(J12&lt;&gt;"",I12&gt;=NOW()),"Planned",IF(AND(J12&lt;&gt;"",J12&lt;NOW()),"Completed","Ongoing")))</f>
-        <v/>
-      </c>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L12" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="M12" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N12" s="45">
         <f>IF(ISBLANK(L12), "", L12*VLOOKUP($F12,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O12" s="45" t="str">
+        <v>0</v>
+      </c>
+      <c r="O12" s="45">
         <f>IF(ISBLANK(M12), "", M12*VLOOKUP($F12,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P12" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="P12" s="44" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="13" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="41">
@@ -7285,30 +7408,48 @@
       </c>
       <c r="C13" s="42" t="str">
         <f>IF(ISBLANK(D13), "", _xlfn.CONCAT("T", TEXT(B13, "0000"), "/", VLOOKUP(D13, Internal!$B$35:C$39, 2, FALSE), IF(OR(D13="QA", D13="Revision"), _xlfn.CONCAT("/", H13), "")))</f>
-        <v/>
-      </c>
-      <c r="D13" s="44"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="44"/>
+        <v>T0003/O</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="44" t="s">
+        <v>30</v>
+      </c>
       <c r="H13" s="43"/>
-      <c r="I13" s="46"/>
-      <c r="J13" s="46"/>
+      <c r="I13" s="46">
+        <v>46125.444444444445</v>
+      </c>
+      <c r="J13" s="46">
+        <v>46125.520833333336</v>
+      </c>
       <c r="K13" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L13" s="47"/>
-      <c r="M13" s="47"/>
-      <c r="N13" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L13" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="M13" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N13" s="45">
         <f>IF(ISBLANK(L13), "", L13*VLOOKUP($F13,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O13" s="45" t="str">
+        <v>0</v>
+      </c>
+      <c r="O13" s="45">
         <f>IF(ISBLANK(M13), "", M13*VLOOKUP($F13,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P13" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="P13" s="44" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="14" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="41">
@@ -7316,30 +7457,48 @@
       </c>
       <c r="C14" s="42" t="str">
         <f>IF(ISBLANK(D14), "", _xlfn.CONCAT("T", TEXT(B14, "0000"), "/", VLOOKUP(D14, Internal!$B$35:C$39, 2, FALSE), IF(OR(D14="QA", D14="Revision"), _xlfn.CONCAT("/", H14), "")))</f>
-        <v/>
-      </c>
-      <c r="D14" s="44"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="44"/>
+        <v>T0004/O</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="44" t="s">
+        <v>30</v>
+      </c>
       <c r="H14" s="43"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="46"/>
+      <c r="I14" s="46">
+        <v>46128.354166666664</v>
+      </c>
+      <c r="J14" s="46">
+        <v>46128.430555555555</v>
+      </c>
       <c r="K14" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L14" s="47"/>
-      <c r="M14" s="47"/>
-      <c r="N14" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L14" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="M14" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N14" s="45">
         <f>IF(ISBLANK(L14), "", L14*VLOOKUP($F14,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O14" s="45" t="str">
+        <v>0</v>
+      </c>
+      <c r="O14" s="45">
         <f>IF(ISBLANK(M14), "", M14*VLOOKUP($F14,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P14" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="P14" s="44" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="15" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="41">
@@ -7347,30 +7506,48 @@
       </c>
       <c r="C15" s="42" t="str">
         <f>IF(ISBLANK(D15), "", _xlfn.CONCAT("T", TEXT(B15, "0000"), "/", VLOOKUP(D15, Internal!$B$35:C$39, 2, FALSE), IF(OR(D15="QA", D15="Revision"), _xlfn.CONCAT("/", H15), "")))</f>
-        <v/>
-      </c>
-      <c r="D15" s="44"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="44"/>
+        <v>T0005/O</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="44" t="s">
+        <v>30</v>
+      </c>
       <c r="H15" s="43"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="46"/>
+      <c r="I15" s="46">
+        <v>46139.444444444445</v>
+      </c>
+      <c r="J15" s="46">
+        <v>46139.520833333336</v>
+      </c>
       <c r="K15" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L15" s="47"/>
-      <c r="M15" s="47"/>
-      <c r="N15" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L15" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="M15" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N15" s="45">
         <f>IF(ISBLANK(L15), "", L15*VLOOKUP($F15,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O15" s="45" t="str">
+        <v>0</v>
+      </c>
+      <c r="O15" s="45">
         <f>IF(ISBLANK(M15), "", M15*VLOOKUP($F15,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P15" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="P15" s="44" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="16" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="41">
@@ -7378,30 +7555,48 @@
       </c>
       <c r="C16" s="42" t="str">
         <f>IF(ISBLANK(D16), "", _xlfn.CONCAT("T", TEXT(B16, "0000"), "/", VLOOKUP(D16, Internal!$B$35:C$39, 2, FALSE), IF(OR(D16="QA", D16="Revision"), _xlfn.CONCAT("/", H16), "")))</f>
-        <v/>
-      </c>
-      <c r="D16" s="44"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="G16" s="44"/>
+        <v>T0006/O</v>
+      </c>
+      <c r="D16" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="44" t="s">
+        <v>30</v>
+      </c>
       <c r="H16" s="43"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="46"/>
+      <c r="I16" s="46">
+        <v>46142.354166666664</v>
+      </c>
+      <c r="J16" s="46">
+        <v>46142.430555555555</v>
+      </c>
       <c r="K16" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L16" s="47"/>
-      <c r="M16" s="47"/>
-      <c r="N16" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L16" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="M16" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N16" s="45">
         <f>IF(ISBLANK(L16), "", L16*VLOOKUP($F16,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O16" s="45" t="str">
+        <v>0</v>
+      </c>
+      <c r="O16" s="45">
         <f>IF(ISBLANK(M16), "", M16*VLOOKUP($F16,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P16" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="P16" s="44" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="17" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="41">
@@ -7409,30 +7604,48 @@
       </c>
       <c r="C17" s="42" t="str">
         <f>IF(ISBLANK(D17), "", _xlfn.CONCAT("T", TEXT(B17, "0000"), "/", VLOOKUP(D17, Internal!$B$35:C$39, 2, FALSE), IF(OR(D17="QA", D17="Revision"), _xlfn.CONCAT("/", H17), "")))</f>
-        <v/>
-      </c>
-      <c r="D17" s="44"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="44"/>
+        <v>T0007/O</v>
+      </c>
+      <c r="D17" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" s="44" t="s">
+        <v>30</v>
+      </c>
       <c r="H17" s="43"/>
-      <c r="I17" s="46"/>
-      <c r="J17" s="46"/>
+      <c r="I17" s="46">
+        <v>46146.444444444445</v>
+      </c>
+      <c r="J17" s="46">
+        <v>46146.520833333336</v>
+      </c>
       <c r="K17" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L17" s="47"/>
-      <c r="M17" s="47"/>
-      <c r="N17" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L17" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="M17" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N17" s="45">
         <f>IF(ISBLANK(L17), "", L17*VLOOKUP($F17,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O17" s="45" t="str">
+        <v>0</v>
+      </c>
+      <c r="O17" s="45">
         <f>IF(ISBLANK(M17), "", M17*VLOOKUP($F17,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P17" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="P17" s="44" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="18" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="41">
@@ -7440,30 +7653,48 @@
       </c>
       <c r="C18" s="42" t="str">
         <f>IF(ISBLANK(D18), "", _xlfn.CONCAT("T", TEXT(B18, "0000"), "/", VLOOKUP(D18, Internal!$B$35:C$39, 2, FALSE), IF(OR(D18="QA", D18="Revision"), _xlfn.CONCAT("/", H18), "")))</f>
-        <v/>
-      </c>
-      <c r="D18" s="44"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="44"/>
+        <v>T0008/O</v>
+      </c>
+      <c r="D18" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="44" t="s">
+        <v>30</v>
+      </c>
       <c r="H18" s="43"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="46"/>
+      <c r="I18" s="46">
+        <v>46119.354166666664</v>
+      </c>
+      <c r="J18" s="46">
+        <v>46119.430555555555</v>
+      </c>
       <c r="K18" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L18" s="47"/>
-      <c r="M18" s="47"/>
-      <c r="N18" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L18" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="M18" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N18" s="45">
         <f>IF(ISBLANK(L18), "", L18*VLOOKUP($F18,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O18" s="45" t="str">
+        <v>0</v>
+      </c>
+      <c r="O18" s="45">
         <f>IF(ISBLANK(M18), "", M18*VLOOKUP($F18,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P18" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="P18" s="44" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="41">
@@ -7471,30 +7702,48 @@
       </c>
       <c r="C19" s="42" t="str">
         <f>IF(ISBLANK(D19), "", _xlfn.CONCAT("T", TEXT(B19, "0000"), "/", VLOOKUP(D19, Internal!$B$35:C$39, 2, FALSE), IF(OR(D19="QA", D19="Revision"), _xlfn.CONCAT("/", H19), "")))</f>
-        <v/>
-      </c>
-      <c r="D19" s="44"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="43"/>
-      <c r="G19" s="44"/>
+        <v>T0009/D</v>
+      </c>
+      <c r="D19" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F19" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="G19" s="44" t="s">
+        <v>37</v>
+      </c>
       <c r="H19" s="43"/>
-      <c r="I19" s="46"/>
-      <c r="J19" s="46"/>
+      <c r="I19" s="46">
+        <v>46124</v>
+      </c>
+      <c r="J19" s="46">
+        <v>46124.999305555553</v>
+      </c>
       <c r="K19" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L19" s="47"/>
-      <c r="M19" s="47"/>
-      <c r="N19" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L19" s="47">
+        <v>1.5</v>
+      </c>
+      <c r="M19" s="47">
+        <v>1</v>
+      </c>
+      <c r="N19" s="45">
         <f>IF(ISBLANK(L19), "", L19*VLOOKUP($F19,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O19" s="45" t="str">
+        <v>60</v>
+      </c>
+      <c r="O19" s="45">
         <f>IF(ISBLANK(M19), "", M19*VLOOKUP($F19,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P19" s="44"/>
+        <v>40</v>
+      </c>
+      <c r="P19" s="44" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="20" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="41">
@@ -7502,30 +7751,48 @@
       </c>
       <c r="C20" s="42" t="str">
         <f>IF(ISBLANK(D20), "", _xlfn.CONCAT("T", TEXT(B20, "0000"), "/", VLOOKUP(D20, Internal!$B$35:C$39, 2, FALSE), IF(OR(D20="QA", D20="Revision"), _xlfn.CONCAT("/", H20), "")))</f>
-        <v/>
-      </c>
-      <c r="D20" s="44"/>
-      <c r="E20" s="43"/>
-      <c r="F20" s="43"/>
-      <c r="G20" s="44"/>
+        <v>T0010/D</v>
+      </c>
+      <c r="D20" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F20" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="G20" s="44" t="s">
+        <v>36</v>
+      </c>
       <c r="H20" s="43"/>
-      <c r="I20" s="46"/>
-      <c r="J20" s="46"/>
+      <c r="I20" s="46">
+        <v>46138</v>
+      </c>
+      <c r="J20" s="46">
+        <v>46139.444444444445</v>
+      </c>
       <c r="K20" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L20" s="47"/>
-      <c r="M20" s="47"/>
-      <c r="N20" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L20" s="47">
+        <v>2.5</v>
+      </c>
+      <c r="M20" s="47">
+        <v>3</v>
+      </c>
+      <c r="N20" s="45">
         <f>IF(ISBLANK(L20), "", L20*VLOOKUP($F20,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O20" s="45" t="str">
+        <v>100</v>
+      </c>
+      <c r="O20" s="45">
         <f>IF(ISBLANK(M20), "", M20*VLOOKUP($F20,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P20" s="44"/>
+        <v>120</v>
+      </c>
+      <c r="P20" s="44" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="21" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="41">
@@ -7533,30 +7800,48 @@
       </c>
       <c r="C21" s="42" t="str">
         <f>IF(ISBLANK(D21), "", _xlfn.CONCAT("T", TEXT(B21, "0000"), "/", VLOOKUP(D21, Internal!$B$35:C$39, 2, FALSE), IF(OR(D21="QA", D21="Revision"), _xlfn.CONCAT("/", H21), "")))</f>
-        <v/>
-      </c>
-      <c r="D21" s="44"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="44"/>
+        <v>T0011/D</v>
+      </c>
+      <c r="D21" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F21" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H21" s="43"/>
-      <c r="I21" s="46"/>
-      <c r="J21" s="46"/>
+      <c r="I21" s="46">
+        <v>46139.520833333336</v>
+      </c>
+      <c r="J21" s="46">
+        <v>46139.999305555553</v>
+      </c>
       <c r="K21" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L21" s="47"/>
-      <c r="M21" s="47"/>
-      <c r="N21" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L21" s="47">
+        <v>0.5</v>
+      </c>
+      <c r="M21" s="47">
+        <v>0.45</v>
+      </c>
+      <c r="N21" s="45">
         <f>IF(ISBLANK(L21), "", L21*VLOOKUP($F21,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O21" s="45" t="str">
+        <v>12.5</v>
+      </c>
+      <c r="O21" s="45">
         <f>IF(ISBLANK(M21), "", M21*VLOOKUP($F21,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P21" s="44"/>
+        <v>11.25</v>
+      </c>
+      <c r="P21" s="44" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="22" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="41">
@@ -7564,30 +7849,48 @@
       </c>
       <c r="C22" s="42" t="str">
         <f>IF(ISBLANK(D22), "", _xlfn.CONCAT("T", TEXT(B22, "0000"), "/", VLOOKUP(D22, Internal!$B$35:C$39, 2, FALSE), IF(OR(D22="QA", D22="Revision"), _xlfn.CONCAT("/", H22), "")))</f>
-        <v/>
-      </c>
-      <c r="D22" s="44"/>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="44"/>
+        <v>T0012/D</v>
+      </c>
+      <c r="D22" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H22" s="43"/>
-      <c r="I22" s="46"/>
-      <c r="J22" s="46"/>
+      <c r="I22" s="46">
+        <v>46139.520833333336</v>
+      </c>
+      <c r="J22" s="46">
+        <v>46140.645833333336</v>
+      </c>
       <c r="K22" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L22" s="47"/>
-      <c r="M22" s="47"/>
-      <c r="N22" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L22" s="47">
+        <v>2.5</v>
+      </c>
+      <c r="M22" s="47">
+        <v>3.15</v>
+      </c>
+      <c r="N22" s="45">
         <f>IF(ISBLANK(L22), "", L22*VLOOKUP($F22,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O22" s="45" t="str">
+        <v>62.5</v>
+      </c>
+      <c r="O22" s="45">
         <f>IF(ISBLANK(M22), "", M22*VLOOKUP($F22,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P22" s="44"/>
+        <v>78.75</v>
+      </c>
+      <c r="P22" s="44" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="23" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="41">
@@ -7595,30 +7898,48 @@
       </c>
       <c r="C23" s="42" t="str">
         <f>IF(ISBLANK(D23), "", _xlfn.CONCAT("T", TEXT(B23, "0000"), "/", VLOOKUP(D23, Internal!$B$35:C$39, 2, FALSE), IF(OR(D23="QA", D23="Revision"), _xlfn.CONCAT("/", H23), "")))</f>
-        <v/>
-      </c>
-      <c r="D23" s="44"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="44"/>
+        <v>T0013/D</v>
+      </c>
+      <c r="D23" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F23" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G23" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H23" s="43"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46"/>
+      <c r="I23" s="46">
+        <v>46140.645833333336</v>
+      </c>
+      <c r="J23" s="46">
+        <v>46140.999305555553</v>
+      </c>
       <c r="K23" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L23" s="47"/>
-      <c r="M23" s="47"/>
-      <c r="N23" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L23" s="47">
+        <v>2</v>
+      </c>
+      <c r="M23" s="47">
+        <v>2.23</v>
+      </c>
+      <c r="N23" s="45">
         <f>IF(ISBLANK(L23), "", L23*VLOOKUP($F23,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O23" s="45" t="str">
+        <v>50</v>
+      </c>
+      <c r="O23" s="45">
         <f>IF(ISBLANK(M23), "", M23*VLOOKUP($F23,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P23" s="44"/>
+        <v>55.75</v>
+      </c>
+      <c r="P23" s="44" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="24" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="41">
@@ -7626,30 +7947,48 @@
       </c>
       <c r="C24" s="42" t="str">
         <f>IF(ISBLANK(D24), "", _xlfn.CONCAT("T", TEXT(B24, "0000"), "/", VLOOKUP(D24, Internal!$B$35:C$39, 2, FALSE), IF(OR(D24="QA", D24="Revision"), _xlfn.CONCAT("/", H24), "")))</f>
-        <v/>
-      </c>
-      <c r="D24" s="44"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="44"/>
+        <v>T0014/D</v>
+      </c>
+      <c r="D24" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F24" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H24" s="43"/>
-      <c r="I24" s="46"/>
-      <c r="J24" s="46"/>
+      <c r="I24" s="46">
+        <v>46140.645833333336</v>
+      </c>
+      <c r="J24" s="46">
+        <v>46140.999305555553</v>
+      </c>
       <c r="K24" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L24" s="47"/>
-      <c r="M24" s="47"/>
-      <c r="N24" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L24" s="47">
+        <v>0.75</v>
+      </c>
+      <c r="M24" s="47">
+        <v>0.51</v>
+      </c>
+      <c r="N24" s="45">
         <f>IF(ISBLANK(L24), "", L24*VLOOKUP($F24,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O24" s="45" t="str">
+        <v>18.75</v>
+      </c>
+      <c r="O24" s="45">
         <f>IF(ISBLANK(M24), "", M24*VLOOKUP($F24,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P24" s="44"/>
+        <v>12.75</v>
+      </c>
+      <c r="P24" s="44" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="25" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="41">
@@ -7657,30 +7996,48 @@
       </c>
       <c r="C25" s="42" t="str">
         <f>IF(ISBLANK(D25), "", _xlfn.CONCAT("T", TEXT(B25, "0000"), "/", VLOOKUP(D25, Internal!$B$35:C$39, 2, FALSE), IF(OR(D25="QA", D25="Revision"), _xlfn.CONCAT("/", H25), "")))</f>
-        <v/>
-      </c>
-      <c r="D25" s="44"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="44"/>
+        <v>T0015/D</v>
+      </c>
+      <c r="D25" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F25" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H25" s="43"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="46"/>
+      <c r="I25" s="46">
+        <v>46139.444444444445</v>
+      </c>
+      <c r="J25" s="46">
+        <v>46139.520833333336</v>
+      </c>
       <c r="K25" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L25" s="47"/>
-      <c r="M25" s="47"/>
-      <c r="N25" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L25" s="47">
+        <v>0.33</v>
+      </c>
+      <c r="M25" s="47">
+        <v>0.25</v>
+      </c>
+      <c r="N25" s="45">
         <f>IF(ISBLANK(L25), "", L25*VLOOKUP($F25,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O25" s="45" t="str">
+        <v>8.25</v>
+      </c>
+      <c r="O25" s="45">
         <f>IF(ISBLANK(M25), "", M25*VLOOKUP($F25,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P25" s="44"/>
+        <v>6.25</v>
+      </c>
+      <c r="P25" s="44" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="26" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="41">
@@ -7688,30 +8045,48 @@
       </c>
       <c r="C26" s="42" t="str">
         <f>IF(ISBLANK(D26), "", _xlfn.CONCAT("T", TEXT(B26, "0000"), "/", VLOOKUP(D26, Internal!$B$35:C$39, 2, FALSE), IF(OR(D26="QA", D26="Revision"), _xlfn.CONCAT("/", H26), "")))</f>
-        <v/>
-      </c>
-      <c r="D26" s="44"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="44"/>
+        <v>T0016/D</v>
+      </c>
+      <c r="D26" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E26" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="F26" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H26" s="43"/>
-      <c r="I26" s="46"/>
-      <c r="J26" s="46"/>
+      <c r="I26" s="46">
+        <v>46139.444444444445</v>
+      </c>
+      <c r="J26" s="46">
+        <v>46139.75</v>
+      </c>
       <c r="K26" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L26" s="47"/>
-      <c r="M26" s="47"/>
-      <c r="N26" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L26" s="47">
+        <v>2</v>
+      </c>
+      <c r="M26" s="47">
+        <v>2.16</v>
+      </c>
+      <c r="N26" s="45">
         <f>IF(ISBLANK(L26), "", L26*VLOOKUP($F26,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O26" s="45" t="str">
+        <v>50</v>
+      </c>
+      <c r="O26" s="45">
         <f>IF(ISBLANK(M26), "", M26*VLOOKUP($F26,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P26" s="44"/>
+        <v>54</v>
+      </c>
+      <c r="P26" s="44" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="27" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="41">
@@ -7719,30 +8094,48 @@
       </c>
       <c r="C27" s="42" t="str">
         <f>IF(ISBLANK(D27), "", _xlfn.CONCAT("T", TEXT(B27, "0000"), "/", VLOOKUP(D27, Internal!$B$35:C$39, 2, FALSE), IF(OR(D27="QA", D27="Revision"), _xlfn.CONCAT("/", H27), "")))</f>
-        <v/>
-      </c>
-      <c r="D27" s="44"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="44"/>
+        <v>T0017/D</v>
+      </c>
+      <c r="D27" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="F27" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H27" s="43"/>
-      <c r="I27" s="46"/>
-      <c r="J27" s="46"/>
+      <c r="I27" s="46">
+        <v>46139.444444444445</v>
+      </c>
+      <c r="J27" s="46">
+        <v>46141.999305555553</v>
+      </c>
       <c r="K27" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L27" s="47"/>
-      <c r="M27" s="47"/>
-      <c r="N27" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L27" s="47">
+        <v>3</v>
+      </c>
+      <c r="M27" s="47">
+        <v>3.33</v>
+      </c>
+      <c r="N27" s="45">
         <f>IF(ISBLANK(L27), "", L27*VLOOKUP($F27,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O27" s="45" t="str">
+        <v>75</v>
+      </c>
+      <c r="O27" s="45">
         <f>IF(ISBLANK(M27), "", M27*VLOOKUP($F27,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P27" s="44"/>
+        <v>83.25</v>
+      </c>
+      <c r="P27" s="44" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="28" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="41">
@@ -7750,30 +8143,48 @@
       </c>
       <c r="C28" s="42" t="str">
         <f>IF(ISBLANK(D28), "", _xlfn.CONCAT("T", TEXT(B28, "0000"), "/", VLOOKUP(D28, Internal!$B$35:C$39, 2, FALSE), IF(OR(D28="QA", D28="Revision"), _xlfn.CONCAT("/", H28), "")))</f>
-        <v/>
-      </c>
-      <c r="D28" s="44"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="44"/>
+        <v>T0018/D</v>
+      </c>
+      <c r="D28" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="F28" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H28" s="43"/>
-      <c r="I28" s="46"/>
-      <c r="J28" s="46"/>
+      <c r="I28" s="46">
+        <v>46139.444444444445</v>
+      </c>
+      <c r="J28" s="46">
+        <v>46144.999305555553</v>
+      </c>
       <c r="K28" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L28" s="47"/>
-      <c r="M28" s="47"/>
-      <c r="N28" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L28" s="47">
+        <v>4.5</v>
+      </c>
+      <c r="M28" s="47">
+        <v>4</v>
+      </c>
+      <c r="N28" s="45">
         <f>IF(ISBLANK(L28), "", L28*VLOOKUP($F28,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O28" s="45" t="str">
+        <v>112.5</v>
+      </c>
+      <c r="O28" s="45">
         <f>IF(ISBLANK(M28), "", M28*VLOOKUP($F28,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P28" s="44"/>
+        <v>100</v>
+      </c>
+      <c r="P28" s="44" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="29" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="41">
@@ -7781,30 +8192,48 @@
       </c>
       <c r="C29" s="42" t="str">
         <f>IF(ISBLANK(D29), "", _xlfn.CONCAT("T", TEXT(B29, "0000"), "/", VLOOKUP(D29, Internal!$B$35:C$39, 2, FALSE), IF(OR(D29="QA", D29="Revision"), _xlfn.CONCAT("/", H29), "")))</f>
-        <v/>
-      </c>
-      <c r="D29" s="44"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="44"/>
+        <v>T0019/D</v>
+      </c>
+      <c r="D29" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F29" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G29" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H29" s="43"/>
-      <c r="I29" s="46"/>
-      <c r="J29" s="46"/>
+      <c r="I29" s="46">
+        <v>46141</v>
+      </c>
+      <c r="J29" s="46">
+        <v>46141.999305555553</v>
+      </c>
       <c r="K29" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L29" s="47"/>
-      <c r="M29" s="47"/>
-      <c r="N29" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L29" s="47">
+        <v>0.83</v>
+      </c>
+      <c r="M29" s="47">
+        <v>0.25</v>
+      </c>
+      <c r="N29" s="45">
         <f>IF(ISBLANK(L29), "", L29*VLOOKUP($F29,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O29" s="45" t="str">
+        <v>20.75</v>
+      </c>
+      <c r="O29" s="45">
         <f>IF(ISBLANK(M29), "", M29*VLOOKUP($F29,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P29" s="44"/>
+        <v>6.25</v>
+      </c>
+      <c r="P29" s="44" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="30" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="41">
@@ -7812,30 +8241,48 @@
       </c>
       <c r="C30" s="42" t="str">
         <f>IF(ISBLANK(D30), "", _xlfn.CONCAT("T", TEXT(B30, "0000"), "/", VLOOKUP(D30, Internal!$B$35:C$39, 2, FALSE), IF(OR(D30="QA", D30="Revision"), _xlfn.CONCAT("/", H30), "")))</f>
-        <v/>
-      </c>
-      <c r="D30" s="44"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="44"/>
+        <v>T0020/D</v>
+      </c>
+      <c r="D30" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E30" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F30" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H30" s="43"/>
-      <c r="I30" s="46"/>
-      <c r="J30" s="46"/>
+      <c r="I30" s="46">
+        <v>46141</v>
+      </c>
+      <c r="J30" s="46">
+        <v>46145.999305555553</v>
+      </c>
       <c r="K30" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L30" s="47"/>
-      <c r="M30" s="47"/>
-      <c r="N30" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L30" s="47">
+        <v>2</v>
+      </c>
+      <c r="M30" s="47">
+        <v>1.53</v>
+      </c>
+      <c r="N30" s="45">
         <f>IF(ISBLANK(L30), "", L30*VLOOKUP($F30,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O30" s="45" t="str">
+        <v>50</v>
+      </c>
+      <c r="O30" s="45">
         <f>IF(ISBLANK(M30), "", M30*VLOOKUP($F30,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P30" s="44"/>
+        <v>38.25</v>
+      </c>
+      <c r="P30" s="44" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="31" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="41">
@@ -7843,30 +8290,48 @@
       </c>
       <c r="C31" s="42" t="str">
         <f>IF(ISBLANK(D31), "", _xlfn.CONCAT("T", TEXT(B31, "0000"), "/", VLOOKUP(D31, Internal!$B$35:C$39, 2, FALSE), IF(OR(D31="QA", D31="Revision"), _xlfn.CONCAT("/", H31), "")))</f>
-        <v/>
-      </c>
-      <c r="D31" s="44"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="44"/>
+        <v>T0021/D</v>
+      </c>
+      <c r="D31" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F31" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H31" s="43"/>
-      <c r="I31" s="46"/>
-      <c r="J31" s="46"/>
+      <c r="I31" s="46">
+        <v>46143</v>
+      </c>
+      <c r="J31" s="46">
+        <v>46145.999305555553</v>
+      </c>
       <c r="K31" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L31" s="47"/>
-      <c r="M31" s="47"/>
-      <c r="N31" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L31" s="47">
+        <v>1</v>
+      </c>
+      <c r="M31" s="47">
+        <v>1</v>
+      </c>
+      <c r="N31" s="45">
         <f>IF(ISBLANK(L31), "", L31*VLOOKUP($F31,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O31" s="45" t="str">
+        <v>25</v>
+      </c>
+      <c r="O31" s="45">
         <f>IF(ISBLANK(M31), "", M31*VLOOKUP($F31,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P31" s="44"/>
+        <v>25</v>
+      </c>
+      <c r="P31" s="44" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="32" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="41">
@@ -7874,30 +8339,48 @@
       </c>
       <c r="C32" s="42" t="str">
         <f>IF(ISBLANK(D32), "", _xlfn.CONCAT("T", TEXT(B32, "0000"), "/", VLOOKUP(D32, Internal!$B$35:C$39, 2, FALSE), IF(OR(D32="QA", D32="Revision"), _xlfn.CONCAT("/", H32), "")))</f>
-        <v/>
-      </c>
-      <c r="D32" s="44"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="44"/>
+        <v>T0022/D</v>
+      </c>
+      <c r="D32" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E32" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F32" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G32" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H32" s="43"/>
-      <c r="I32" s="46"/>
-      <c r="J32" s="46"/>
+      <c r="I32" s="46">
+        <v>46143</v>
+      </c>
+      <c r="J32" s="46">
+        <v>46145.999305555553</v>
+      </c>
       <c r="K32" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L32" s="47"/>
-      <c r="M32" s="47"/>
-      <c r="N32" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L32" s="47">
+        <v>1.5</v>
+      </c>
+      <c r="M32" s="47">
+        <v>0.8</v>
+      </c>
+      <c r="N32" s="45">
         <f>IF(ISBLANK(L32), "", L32*VLOOKUP($F32,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O32" s="45" t="str">
+        <v>37.5</v>
+      </c>
+      <c r="O32" s="45">
         <f>IF(ISBLANK(M32), "", M32*VLOOKUP($F32,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P32" s="44"/>
+        <v>20</v>
+      </c>
+      <c r="P32" s="44" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="33" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="41">
@@ -7905,30 +8388,48 @@
       </c>
       <c r="C33" s="42" t="str">
         <f>IF(ISBLANK(D33), "", _xlfn.CONCAT("T", TEXT(B33, "0000"), "/", VLOOKUP(D33, Internal!$B$35:C$39, 2, FALSE), IF(OR(D33="QA", D33="Revision"), _xlfn.CONCAT("/", H33), "")))</f>
-        <v/>
-      </c>
-      <c r="D33" s="44"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="44"/>
+        <v>T0023/D</v>
+      </c>
+      <c r="D33" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E33" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F33" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G33" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H33" s="43"/>
-      <c r="I33" s="46"/>
-      <c r="J33" s="46"/>
+      <c r="I33" s="46">
+        <v>46143</v>
+      </c>
+      <c r="J33" s="46">
+        <v>46145</v>
+      </c>
       <c r="K33" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L33" s="47"/>
-      <c r="M33" s="47"/>
-      <c r="N33" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L33" s="47">
+        <v>1.5</v>
+      </c>
+      <c r="M33" s="47">
+        <v>1.58</v>
+      </c>
+      <c r="N33" s="45">
         <f>IF(ISBLANK(L33), "", L33*VLOOKUP($F33,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O33" s="45" t="str">
+        <v>37.5</v>
+      </c>
+      <c r="O33" s="45">
         <f>IF(ISBLANK(M33), "", M33*VLOOKUP($F33,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P33" s="44"/>
+        <v>39.5</v>
+      </c>
+      <c r="P33" s="44" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="34" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="41">
@@ -7936,30 +8437,48 @@
       </c>
       <c r="C34" s="42" t="str">
         <f>IF(ISBLANK(D34), "", _xlfn.CONCAT("T", TEXT(B34, "0000"), "/", VLOOKUP(D34, Internal!$B$35:C$39, 2, FALSE), IF(OR(D34="QA", D34="Revision"), _xlfn.CONCAT("/", H34), "")))</f>
-        <v/>
-      </c>
-      <c r="D34" s="44"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="44"/>
+        <v>T0024/D</v>
+      </c>
+      <c r="D34" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E34" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="F34" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H34" s="43"/>
-      <c r="I34" s="46"/>
-      <c r="J34" s="46"/>
+      <c r="I34" s="46">
+        <v>46141</v>
+      </c>
+      <c r="J34" s="46">
+        <v>46141.999305555553</v>
+      </c>
       <c r="K34" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L34" s="47"/>
-      <c r="M34" s="47"/>
-      <c r="N34" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L34" s="47">
+        <v>2</v>
+      </c>
+      <c r="M34" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N34" s="45">
         <f>IF(ISBLANK(L34), "", L34*VLOOKUP($F34,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O34" s="45" t="str">
+        <v>50</v>
+      </c>
+      <c r="O34" s="45">
         <f>IF(ISBLANK(M34), "", M34*VLOOKUP($F34,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P34" s="44"/>
+        <v>45.75</v>
+      </c>
+      <c r="P34" s="44" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="35" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="41">
@@ -7967,30 +8486,48 @@
       </c>
       <c r="C35" s="42" t="str">
         <f>IF(ISBLANK(D35), "", _xlfn.CONCAT("T", TEXT(B35, "0000"), "/", VLOOKUP(D35, Internal!$B$35:C$39, 2, FALSE), IF(OR(D35="QA", D35="Revision"), _xlfn.CONCAT("/", H35), "")))</f>
-        <v/>
-      </c>
-      <c r="D35" s="44"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="44"/>
+        <v>T0025/D</v>
+      </c>
+      <c r="D35" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E35" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="F35" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G35" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H35" s="43"/>
-      <c r="I35" s="46"/>
-      <c r="J35" s="46"/>
+      <c r="I35" s="46">
+        <v>46142</v>
+      </c>
+      <c r="J35" s="46">
+        <v>46142.999305555553</v>
+      </c>
       <c r="K35" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L35" s="47"/>
-      <c r="M35" s="47"/>
-      <c r="N35" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L35" s="47">
+        <v>1</v>
+      </c>
+      <c r="M35" s="47">
+        <v>1.18</v>
+      </c>
+      <c r="N35" s="45">
         <f>IF(ISBLANK(L35), "", L35*VLOOKUP($F35,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O35" s="45" t="str">
+        <v>25</v>
+      </c>
+      <c r="O35" s="45">
         <f>IF(ISBLANK(M35), "", M35*VLOOKUP($F35,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P35" s="44"/>
+        <v>29.5</v>
+      </c>
+      <c r="P35" s="44" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="36" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="41">
@@ -7998,30 +8535,48 @@
       </c>
       <c r="C36" s="42" t="str">
         <f>IF(ISBLANK(D36), "", _xlfn.CONCAT("T", TEXT(B36, "0000"), "/", VLOOKUP(D36, Internal!$B$35:C$39, 2, FALSE), IF(OR(D36="QA", D36="Revision"), _xlfn.CONCAT("/", H36), "")))</f>
-        <v/>
-      </c>
-      <c r="D36" s="44"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="44"/>
+        <v>T0026/D</v>
+      </c>
+      <c r="D36" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E36" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="F36" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G36" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H36" s="43"/>
-      <c r="I36" s="46"/>
-      <c r="J36" s="46"/>
+      <c r="I36" s="46">
+        <v>46145</v>
+      </c>
+      <c r="J36" s="46">
+        <v>46145.999305555553</v>
+      </c>
       <c r="K36" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L36" s="47"/>
-      <c r="M36" s="47"/>
-      <c r="N36" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L36" s="47">
+        <v>4</v>
+      </c>
+      <c r="M36" s="47">
+        <v>5.38</v>
+      </c>
+      <c r="N36" s="45">
         <f>IF(ISBLANK(L36), "", L36*VLOOKUP($F36,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O36" s="45" t="str">
+        <v>100</v>
+      </c>
+      <c r="O36" s="45">
         <f>IF(ISBLANK(M36), "", M36*VLOOKUP($F36,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P36" s="44"/>
+        <v>134.5</v>
+      </c>
+      <c r="P36" s="44" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="37" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="41">
@@ -8029,30 +8584,48 @@
       </c>
       <c r="C37" s="42" t="str">
         <f>IF(ISBLANK(D37), "", _xlfn.CONCAT("T", TEXT(B37, "0000"), "/", VLOOKUP(D37, Internal!$B$35:C$39, 2, FALSE), IF(OR(D37="QA", D37="Revision"), _xlfn.CONCAT("/", H37), "")))</f>
-        <v/>
-      </c>
-      <c r="D37" s="44"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="44"/>
+        <v>T0027/D</v>
+      </c>
+      <c r="D37" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E37" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="F37" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G37" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H37" s="43"/>
-      <c r="I37" s="46"/>
-      <c r="J37" s="46"/>
+      <c r="I37" s="46">
+        <v>46139.520833333336</v>
+      </c>
+      <c r="J37" s="46">
+        <v>46143.999305555553</v>
+      </c>
       <c r="K37" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L37" s="47"/>
-      <c r="M37" s="47"/>
-      <c r="N37" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L37" s="47">
+        <v>2</v>
+      </c>
+      <c r="M37" s="47">
+        <v>1.83</v>
+      </c>
+      <c r="N37" s="45">
         <f>IF(ISBLANK(L37), "", L37*VLOOKUP($F37,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O37" s="45" t="str">
+        <v>50</v>
+      </c>
+      <c r="O37" s="45">
         <f>IF(ISBLANK(M37), "", M37*VLOOKUP($F37,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P37" s="44"/>
+        <v>45.75</v>
+      </c>
+      <c r="P37" s="44" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="38" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="41">
@@ -8060,30 +8633,48 @@
       </c>
       <c r="C38" s="42" t="str">
         <f>IF(ISBLANK(D38), "", _xlfn.CONCAT("T", TEXT(B38, "0000"), "/", VLOOKUP(D38, Internal!$B$35:C$39, 2, FALSE), IF(OR(D38="QA", D38="Revision"), _xlfn.CONCAT("/", H38), "")))</f>
-        <v/>
-      </c>
-      <c r="D38" s="44"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="44"/>
+        <v>T0028/D</v>
+      </c>
+      <c r="D38" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E38" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="F38" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G38" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H38" s="43"/>
-      <c r="I38" s="46"/>
-      <c r="J38" s="46"/>
+      <c r="I38" s="46">
+        <v>46143</v>
+      </c>
+      <c r="J38" s="46">
+        <v>46145.999305555553</v>
+      </c>
       <c r="K38" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L38" s="47"/>
-      <c r="M38" s="47"/>
-      <c r="N38" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L38" s="47">
+        <v>2</v>
+      </c>
+      <c r="M38" s="47">
+        <v>1.55</v>
+      </c>
+      <c r="N38" s="45">
         <f>IF(ISBLANK(L38), "", L38*VLOOKUP($F38,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O38" s="45" t="str">
+        <v>50</v>
+      </c>
+      <c r="O38" s="45">
         <f>IF(ISBLANK(M38), "", M38*VLOOKUP($F38,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P38" s="44"/>
+        <v>38.75</v>
+      </c>
+      <c r="P38" s="44" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="39" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="41">
@@ -8091,30 +8682,48 @@
       </c>
       <c r="C39" s="42" t="str">
         <f>IF(ISBLANK(D39), "", _xlfn.CONCAT("T", TEXT(B39, "0000"), "/", VLOOKUP(D39, Internal!$B$35:C$39, 2, FALSE), IF(OR(D39="QA", D39="Revision"), _xlfn.CONCAT("/", H39), "")))</f>
-        <v/>
-      </c>
-      <c r="D39" s="44"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="44"/>
+        <v>T0029/D</v>
+      </c>
+      <c r="D39" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E39" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="F39" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G39" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H39" s="43"/>
-      <c r="I39" s="46"/>
-      <c r="J39" s="46"/>
+      <c r="I39" s="46">
+        <v>46146</v>
+      </c>
+      <c r="J39" s="46">
+        <v>46146.999305555553</v>
+      </c>
       <c r="K39" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L39" s="47"/>
-      <c r="M39" s="47"/>
-      <c r="N39" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L39" s="47">
+        <v>1.5</v>
+      </c>
+      <c r="M39" s="47">
+        <v>1.25</v>
+      </c>
+      <c r="N39" s="45">
         <f>IF(ISBLANK(L39), "", L39*VLOOKUP($F39,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O39" s="45" t="str">
+        <v>37.5</v>
+      </c>
+      <c r="O39" s="45">
         <f>IF(ISBLANK(M39), "", M39*VLOOKUP($F39,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P39" s="44"/>
+        <v>31.25</v>
+      </c>
+      <c r="P39" s="44" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="40" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="41">
@@ -8122,30 +8731,48 @@
       </c>
       <c r="C40" s="42" t="str">
         <f>IF(ISBLANK(D40), "", _xlfn.CONCAT("T", TEXT(B40, "0000"), "/", VLOOKUP(D40, Internal!$B$35:C$39, 2, FALSE), IF(OR(D40="QA", D40="Revision"), _xlfn.CONCAT("/", H40), "")))</f>
-        <v/>
-      </c>
-      <c r="D40" s="44"/>
-      <c r="E40" s="43"/>
-      <c r="F40" s="43"/>
-      <c r="G40" s="44"/>
+        <v>T0030/D</v>
+      </c>
+      <c r="D40" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E40" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="F40" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G40" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H40" s="43"/>
-      <c r="I40" s="46"/>
-      <c r="J40" s="46"/>
+      <c r="I40" s="46">
+        <v>46143</v>
+      </c>
+      <c r="J40" s="46">
+        <v>46143.999305555553</v>
+      </c>
       <c r="K40" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L40" s="47"/>
-      <c r="M40" s="47"/>
-      <c r="N40" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L40" s="47">
+        <v>1.5</v>
+      </c>
+      <c r="M40" s="47">
+        <v>1.55</v>
+      </c>
+      <c r="N40" s="45">
         <f>IF(ISBLANK(L40), "", L40*VLOOKUP($F40,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O40" s="45" t="str">
+        <v>37.5</v>
+      </c>
+      <c r="O40" s="45">
         <f>IF(ISBLANK(M40), "", M40*VLOOKUP($F40,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P40" s="44"/>
+        <v>38.75</v>
+      </c>
+      <c r="P40" s="44" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="41" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="41">
@@ -8153,30 +8780,48 @@
       </c>
       <c r="C41" s="42" t="str">
         <f>IF(ISBLANK(D41), "", _xlfn.CONCAT("T", TEXT(B41, "0000"), "/", VLOOKUP(D41, Internal!$B$35:C$39, 2, FALSE), IF(OR(D41="QA", D41="Revision"), _xlfn.CONCAT("/", H41), "")))</f>
-        <v/>
-      </c>
-      <c r="D41" s="44"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="44"/>
+        <v>T0031/D</v>
+      </c>
+      <c r="D41" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E41" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="F41" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G41" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H41" s="43"/>
-      <c r="I41" s="46"/>
-      <c r="J41" s="46"/>
+      <c r="I41" s="46">
+        <v>46144</v>
+      </c>
+      <c r="J41" s="46">
+        <v>46144.999305555553</v>
+      </c>
       <c r="K41" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L41" s="47"/>
-      <c r="M41" s="47"/>
-      <c r="N41" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L41" s="47">
+        <v>2</v>
+      </c>
+      <c r="M41" s="47">
+        <v>2.5</v>
+      </c>
+      <c r="N41" s="45">
         <f>IF(ISBLANK(L41), "", L41*VLOOKUP($F41,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O41" s="45" t="str">
+        <v>50</v>
+      </c>
+      <c r="O41" s="45">
         <f>IF(ISBLANK(M41), "", M41*VLOOKUP($F41,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P41" s="44"/>
+        <v>62.5</v>
+      </c>
+      <c r="P41" s="44" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="42" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="41">
@@ -8184,30 +8829,48 @@
       </c>
       <c r="C42" s="42" t="str">
         <f>IF(ISBLANK(D42), "", _xlfn.CONCAT("T", TEXT(B42, "0000"), "/", VLOOKUP(D42, Internal!$B$35:C$39, 2, FALSE), IF(OR(D42="QA", D42="Revision"), _xlfn.CONCAT("/", H42), "")))</f>
-        <v/>
-      </c>
-      <c r="D42" s="44"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="44"/>
+        <v>T0032/D</v>
+      </c>
+      <c r="D42" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E42" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="F42" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G42" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H42" s="43"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46"/>
+      <c r="I42" s="46">
+        <v>46146</v>
+      </c>
+      <c r="J42" s="46">
+        <v>46146.999305555553</v>
+      </c>
       <c r="K42" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L42" s="47"/>
-      <c r="M42" s="47"/>
-      <c r="N42" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L42" s="47">
+        <v>1.5</v>
+      </c>
+      <c r="M42" s="47">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="N42" s="45">
         <f>IF(ISBLANK(L42), "", L42*VLOOKUP($F42,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O42" s="45" t="str">
+        <v>37.5</v>
+      </c>
+      <c r="O42" s="45">
         <f>IF(ISBLANK(M42), "", M42*VLOOKUP($F42,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="P42" s="44"/>
+        <v>28.749999999999996</v>
+      </c>
+      <c r="P42" s="44" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="43" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="41">
@@ -8215,12 +8878,20 @@
       </c>
       <c r="C43" s="42" t="str">
         <f>IF(ISBLANK(D43), "", _xlfn.CONCAT("T", TEXT(B43, "0000"), "/", VLOOKUP(D43, Internal!$B$35:C$39, 2, FALSE), IF(OR(D43="QA", D43="Revision"), _xlfn.CONCAT("/", H43), "")))</f>
-        <v/>
-      </c>
-      <c r="D43" s="44"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="43"/>
-      <c r="G43" s="44"/>
+        <v>T0033/D</v>
+      </c>
+      <c r="D43" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E43" s="43" t="s">
+        <v>82</v>
+      </c>
+      <c r="F43" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G43" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="H43" s="43"/>
       <c r="I43" s="46"/>
       <c r="J43" s="46"/>

</xml_diff>